<commit_message>
Flujo de efectivo sin transacciones sin efectivo, demo determinista, autoprueba y empaquetado verificado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UKpqBxWMxzkmJmMnUb2UZS
</commit_message>
<xml_diff>
--- a/ContaBolPy/docs/img/ejemplo_balance_general.xlsx
+++ b/ContaBolPy/docs/img/ejemplo_balance_general.xlsx
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>2259077.83</v>
+        <v>1940499.67</v>
       </c>
     </row>
     <row r="12">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2004249.14</v>
+        <v>1376082.87</v>
       </c>
     </row>
     <row r="13">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>-467379.09</v>
+        <v>-391293.67</v>
       </c>
     </row>
     <row r="14">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B14" s="15" t="n">
-        <v>-467379.09</v>
+        <v>-391293.67</v>
       </c>
     </row>
     <row r="15">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>2471628.23</v>
+        <v>1767376.54</v>
       </c>
     </row>
     <row r="16">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B16" s="15" t="n">
-        <v>2471628.23</v>
+        <v>1767376.54</v>
       </c>
     </row>
     <row r="17">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>44356.84</v>
+        <v>106161.9</v>
       </c>
     </row>
     <row r="18">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>44356.84</v>
+        <v>106161.9</v>
       </c>
     </row>
     <row r="19">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>44356.84</v>
+        <v>106161.9</v>
       </c>
     </row>
     <row r="20">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>210471.85</v>
+        <v>458254.9</v>
       </c>
     </row>
     <row r="21">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>210471.85</v>
+        <v>458254.9</v>
       </c>
     </row>
     <row r="22">
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B22" s="15" t="n">
-        <v>210471.85</v>
+        <v>458254.9</v>
       </c>
     </row>
     <row r="23">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B31" s="19" t="n">
-        <v>2366961.17</v>
+        <v>2048383.01</v>
       </c>
     </row>
     <row r="32">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B33" s="10" t="n">
-        <v>502314.23</v>
+        <v>310971.58</v>
       </c>
     </row>
     <row r="34">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B34" s="10" t="n">
-        <v>233989.24</v>
+        <v>56324.22</v>
       </c>
     </row>
     <row r="35">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>233989.24</v>
+        <v>56324.22</v>
       </c>
     </row>
     <row r="36">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="B36" s="15" t="n">
-        <v>233989.24</v>
+        <v>56324.22</v>
       </c>
     </row>
     <row r="37">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B37" s="10" t="n">
-        <v>139595.89</v>
+        <v>125918.26</v>
       </c>
     </row>
     <row r="38">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="B38" s="15" t="n">
-        <v>139595.89</v>
+        <v>125918.26</v>
       </c>
     </row>
     <row r="39">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>139595.89</v>
+        <v>125918.26</v>
       </c>
     </row>
     <row r="40">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="B51" s="19" t="n">
-        <v>586314.23</v>
+        <v>394971.58</v>
       </c>
     </row>
     <row r="52">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>631346.9399999999</v>
+        <v>504111.43</v>
       </c>
     </row>
     <row r="58">
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B58" s="19" t="n">
-        <v>1780646.94</v>
+        <v>1653411.43</v>
       </c>
     </row>
     <row r="59">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="B59" s="19" t="n">
-        <v>2366961.17</v>
+        <v>2048383.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>